<commit_message>
feat: add JOYCE2810 proprietor admin security lock screen and server-level lead deletion
</commit_message>
<xml_diff>
--- a/server/data/RVS_Leads.xlsx
+++ b/server/data/RVS_Leads.xlsx
@@ -439,34 +439,34 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>16/8/2026, 4:45:50 pm</v>
+        <v>16/8/2026, 4:47:31 pm</v>
       </c>
       <c r="C2" t="str">
-        <v>Sample Demo Lead (RVS Interior)</v>
+        <v>Sundar Pichai</v>
       </c>
       <c r="D2" t="str">
-        <v>9710453183</v>
+        <v>9876543210</v>
       </c>
       <c r="E2" t="str">
-        <v>rvsinterior28@gmail.com</v>
+        <v>sundar@google.com</v>
       </c>
       <c r="F2" t="str">
-        <v>Arumbakkam, Chennai</v>
+        <v>Anna Nagar, Chennai</v>
       </c>
       <c r="G2" t="str">
-        <v>Turnkey Interior Design</v>
+        <v>Full Villa Turnkey Renovation</v>
       </c>
       <c r="H2" t="str">
-        <v>3 BHK</v>
+        <v>4 BHK Villa</v>
       </c>
       <c r="I2" t="str">
-        <v>₹ 4,50,000</v>
+        <v>Rs 15,00,000</v>
       </c>
       <c r="J2" t="str">
-        <v>Interested in Modular Kitchen and False Ceiling under R. Stephen direct supervision.</v>
+        <v>Requirement for premium Italian kitchen and marine plywood wardrobes</v>
       </c>
       <c r="K2" t="str">
-        <v>Website Initializer</v>
+        <v>Website Form</v>
       </c>
     </row>
     <row r="3">
@@ -474,34 +474,34 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>16/8/2026, 4:47:31 pm</v>
+        <v>16/8/2026, 5:03:37 pm</v>
       </c>
       <c r="C3" t="str">
-        <v>Sundar Pichai</v>
+        <v>RAMESH Mino</v>
       </c>
       <c r="D3" t="str">
-        <v>9876543210</v>
+        <v>3566456449</v>
       </c>
       <c r="E3" t="str">
-        <v>sundar@google.com</v>
+        <v>rameshpec28@gmail.com</v>
       </c>
       <c r="F3" t="str">
-        <v>Anna Nagar, Chennai</v>
+        <v>gchgfhjf</v>
       </c>
       <c r="G3" t="str">
-        <v>Full Villa Turnkey Renovation</v>
+        <v>Interior Design</v>
       </c>
       <c r="H3" t="str">
-        <v>4 BHK Villa</v>
+        <v>2 BHK Home</v>
       </c>
       <c r="I3" t="str">
-        <v>Rs 15,00,000</v>
+        <v>₹6,58,800</v>
       </c>
       <c r="J3" t="str">
-        <v>Requirement for premium Italian kitchen and marine plywood wardrobes</v>
+        <v>Calculated from Website Estimator: 2 BHK Home (1050 sq.ft) with Premium finish. Estimated total budget: ₹6,58,800. Please schedule a free site laser measurement.</v>
       </c>
       <c r="K3" t="str">
-        <v>Website Form</v>
+        <v>Website Lead Form</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update admin password placeholder and publish
</commit_message>
<xml_diff>
--- a/server/data/RVS_Leads.xlsx
+++ b/server/data/RVS_Leads.xlsx
@@ -397,116 +397,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K3"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>S.No</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Submitted Date &amp; Time</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Client Name</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Mobile Number</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Email Address</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Chennai Location</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Service Requested</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Property Type</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Estimated Budget</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Client Notes / Requirements</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Lead Source</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="str">
-        <v>16/8/2026, 4:47:31 pm</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Sundar Pichai</v>
-      </c>
-      <c r="D2" t="str">
-        <v>9876543210</v>
-      </c>
-      <c r="E2" t="str">
-        <v>sundar@google.com</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Anna Nagar, Chennai</v>
-      </c>
-      <c r="G2" t="str">
-        <v>Full Villa Turnkey Renovation</v>
-      </c>
-      <c r="H2" t="str">
-        <v>4 BHK Villa</v>
-      </c>
-      <c r="I2" t="str">
-        <v>Rs 15,00,000</v>
-      </c>
-      <c r="J2" t="str">
-        <v>Requirement for premium Italian kitchen and marine plywood wardrobes</v>
-      </c>
-      <c r="K2" t="str">
-        <v>Website Form</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>16/8/2026, 5:03:37 pm</v>
-      </c>
-      <c r="C3" t="str">
-        <v>RAMESH Mino</v>
-      </c>
-      <c r="D3" t="str">
-        <v>3566456449</v>
-      </c>
-      <c r="E3" t="str">
-        <v>rameshpec28@gmail.com</v>
-      </c>
-      <c r="F3" t="str">
-        <v>gchgfhjf</v>
-      </c>
-      <c r="G3" t="str">
-        <v>Interior Design</v>
-      </c>
-      <c r="H3" t="str">
-        <v>2 BHK Home</v>
-      </c>
-      <c r="I3" t="str">
-        <v>₹6,58,800</v>
-      </c>
-      <c r="J3" t="str">
-        <v>Calculated from Website Estimator: 2 BHK Home (1050 sq.ft) with Premium finish. Estimated total budget: ₹6,58,800. Please schedule a free site laser measurement.</v>
-      </c>
-      <c r="K3" t="str">
-        <v>Website Lead Form</v>
-      </c>
-    </row>
-  </sheetData>
+  <dimension ref="A1"/>
+  <sheetData/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>